<commit_message>
Godkendelse af MADS tilføjet til oversigt
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287F6D3B-3F63-47BF-976A-738990663510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BABEF6E-48F1-4136-A5FA-2B67DDA725D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30855" yWindow="1950" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 19-12-2025" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 29-01-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 19-12-2025'!$A$1:$G$2867</definedName>
+    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 29-01-2026'!$A$1:$G$2867</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -33575,7 +33575,7 @@
         <v>15</v>
       </c>
       <c r="G1370" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1371" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Opdateret testresultat til Godkendt for MinGraviditet
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BABEF6E-48F1-4136-A5FA-2B67DDA725D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84E61A3-6634-4737-B9C5-5D47B9A2F02A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 29-01-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 02-02-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 29-01-2026'!$A$1:$G$2867</definedName>
+    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 02-02-2026'!$A$1:$G$2867</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -34242,7 +34242,7 @@
         <v>11</v>
       </c>
       <c r="G1399" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1400" spans="1:7" x14ac:dyDescent="0.25">
@@ -34265,7 +34265,7 @@
         <v>11</v>
       </c>
       <c r="G1400" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1401" spans="1:7" x14ac:dyDescent="0.25">
@@ -34288,7 +34288,7 @@
         <v>11</v>
       </c>
       <c r="G1401" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1402" spans="1:7" x14ac:dyDescent="0.25">
@@ -34311,7 +34311,7 @@
         <v>11</v>
       </c>
       <c r="G1402" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1403" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Versionsnummer for DGB opdateret, så der kun står 0.91 og ikke 0.91 0.91
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D78E85-9BC5-43D7-B89C-DE7F595ABAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A1F51D-6FDB-4A79-AFB9-92A1B9424AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15045" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 10-04-2026" sheetId="1" r:id="rId1"/>
@@ -1379,8 +1379,7 @@
     <t>Den Gode Blanketservice</t>
   </si>
   <si>
-    <t>DGB (0.91_x000D_
-0.91)</t>
+    <t>DGB (0.91)</t>
   </si>
   <si>
     <t>Den Dynamiske Blanket</t>

</xml_diff>

<commit_message>
OS2 ændret til Digital Identity
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A8EE47-3DA6-43E0-AEAA-53143D10C996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31FEF371-0742-4263-823D-8410C8478D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 01-06-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 02-06-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 01-06-2026'!$A$1:$G$2969</definedName>
+    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 02-06-2026'!$A$1:$G$2969</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -1451,7 +1451,7 @@
     <t>OS2korrespondance</t>
   </si>
   <si>
-    <t>OS2</t>
+    <t>Digital Identity</t>
   </si>
   <si>
     <t>Patologi</t>

</xml_diff>

<commit_message>
HejDoktor og BCC godkendelse
HejDoktor og BCC godkendelse.
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hua\GitHub\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0D5892-AD50-4DF7-84A5-2B0D799D98AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A172A1-790B-49A9-BEE5-01D33A7F6096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3150" yWindow="3135" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Opdateret d. 09-06-2026" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Modulus har fået status Godkendt for CC og ACK.
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8580A3F6-11EF-48DD-92B6-7F9AFB46694B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217750D6-8757-4A77-947C-BCE46A54E30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 03-07-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 09-07-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 03-07-2026'!$A$1:$G$3038</definedName>
+    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 09-07-2026'!$A$1:$G$3038</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -37735,7 +37735,7 @@
         <v>18</v>
       </c>
       <c r="G1549" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1550" spans="1:7" x14ac:dyDescent="0.3">
@@ -37781,7 +37781,7 @@
         <v>18</v>
       </c>
       <c r="G1551" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1552" spans="1:7" x14ac:dyDescent="0.3">
@@ -37804,7 +37804,7 @@
         <v>11</v>
       </c>
       <c r="G1552" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1553" spans="1:7" x14ac:dyDescent="0.3">
@@ -37827,7 +37827,7 @@
         <v>18</v>
       </c>
       <c r="G1553" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1554" spans="1:7" x14ac:dyDescent="0.3">
@@ -37965,7 +37965,7 @@
         <v>11</v>
       </c>
       <c r="G1559" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1560" spans="1:7" x14ac:dyDescent="0.3">
@@ -37988,7 +37988,7 @@
         <v>18</v>
       </c>
       <c r="G1560" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1561" spans="1:7" x14ac:dyDescent="0.3">
@@ -38034,7 +38034,7 @@
         <v>11</v>
       </c>
       <c r="G1562" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1563" spans="1:7" x14ac:dyDescent="0.3">
@@ -38057,7 +38057,7 @@
         <v>11</v>
       </c>
       <c r="G1563" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1564" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Vena har fået status Godkendt for afsendelse af DIS13
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217750D6-8757-4A77-947C-BCE46A54E30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27619FAE-BFFC-467F-87A7-EFDF20893131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Opdateret d. 09-07-2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Opdateret d. 19-08-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 09-07-2026'!$A$1:$G$3038</definedName>
+    <definedName name="Alle_systemer__Samlet_liste_">'Opdateret d. 19-08-2026'!$A$1:$G$3038</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -62207,7 +62207,7 @@
         <v>11</v>
       </c>
       <c r="G2613" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2614" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>